<commit_message>
update 2026-06-17: backlog monitoring, MOM, and sprint report outputs
- backlog-monitoring-mkp-implementation: update html & pdf
- MOM BUMA BTECH Digiman+ Product Grooming: update xlsx
- Sprint report outputs: add 20260612, 20260615 html/md/pdf and delayed ticket report

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BUMA-ID-project/mom/MOM - BUMA - BTECH - Digiman+ Product Grooming.xlsx
+++ b/BUMA-ID-project/mom/MOM - BUMA - BTECH - Digiman+ Product Grooming.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bukittech-my.sharepoint.com/personal/okky_rrohayat_bukittechnology_com/Documents/Notebooks/office-notes/BUMA-ID-project/mom/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="11_6B586B98E5D70189ECD1F1651EF943745F0AB558" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9201970-5939-444C-B088-0C55218DB6DB}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="11_6B586B98E5D70189ECD1F1651EF943745F0AB558" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFFAA71E-3CF2-4A2A-8D88-25BAB5607066}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1393,10 +1393,10 @@
     <t>Priority of Product Journey</t>
   </si>
   <si>
-    <t>Yang menjadi prioritas development adalah service sheet (PSCS), baru kemudian form approval, dan seterusnya.</t>
-  </si>
-  <si>
     <t>BUMA, BTECH</t>
+  </si>
+  <si>
+    <t>Yang menjadi prioritas development adalah service sheet (PSCS), baru kemudian form approval, dan Equipment Area.</t>
   </si>
 </sst>
 </file>
@@ -1794,8 +1794,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1803,6 +1803,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1814,9 +1817,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1824,16 +1824,16 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2479,7 +2479,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="82"/>
@@ -2573,25 +2573,25 @@
     <row r="6" spans="1:13" ht="151.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19"/>
       <c r="B6" s="19"/>
-      <c r="C6" s="79" t="s">
+      <c r="C6" s="80" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="78"/>
+      <c r="D6" s="79"/>
       <c r="E6" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="F6" s="77" t="s">
+      <c r="F6" s="78" t="s">
         <v>81</v>
       </c>
-      <c r="G6" s="78"/>
-      <c r="H6" s="78"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="79"/>
       <c r="I6" s="23"/>
-      <c r="J6" s="80"/>
+      <c r="J6" s="81"/>
       <c r="K6" s="83"/>
       <c r="M6" s="5"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="81" t="s">
+      <c r="A7" s="73" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="82"/>
@@ -3219,7 +3219,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="74"/>
@@ -3318,26 +3318,26 @@
     <row r="6" spans="1:13" ht="151.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19"/>
       <c r="B6" s="19"/>
-      <c r="C6" s="79" t="s">
+      <c r="C6" s="80" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="78"/>
+      <c r="D6" s="79"/>
       <c r="E6" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="F6" s="77" t="s">
+      <c r="F6" s="78" t="s">
         <v>127</v>
       </c>
-      <c r="G6" s="78"/>
-      <c r="H6" s="78"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="79"/>
       <c r="I6" s="23"/>
-      <c r="J6" s="80"/>
+      <c r="J6" s="81"/>
       <c r="K6" s="74"/>
       <c r="L6" s="20"/>
       <c r="M6" s="5"/>
     </row>
     <row r="7" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="81" t="s">
+      <c r="A7" s="73" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="74"/>
@@ -4095,7 +4095,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="74"/>
@@ -4194,26 +4194,26 @@
     <row r="6" spans="1:13" ht="151.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19"/>
       <c r="B6" s="19"/>
-      <c r="C6" s="79" t="s">
+      <c r="C6" s="80" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="78"/>
+      <c r="D6" s="79"/>
       <c r="E6" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="F6" s="77" t="s">
+      <c r="F6" s="78" t="s">
         <v>139</v>
       </c>
-      <c r="G6" s="78"/>
-      <c r="H6" s="78"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="79"/>
       <c r="I6" s="23"/>
-      <c r="J6" s="80"/>
+      <c r="J6" s="81"/>
       <c r="K6" s="74"/>
       <c r="L6" s="20"/>
       <c r="M6" s="5"/>
     </row>
     <row r="7" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="81" t="s">
+      <c r="A7" s="73" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="74"/>
@@ -5271,7 +5271,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="74"/>
@@ -5370,26 +5370,26 @@
     <row r="6" spans="1:13" ht="151.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19"/>
       <c r="B6" s="19"/>
-      <c r="C6" s="79" t="s">
+      <c r="C6" s="80" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="78"/>
+      <c r="D6" s="79"/>
       <c r="E6" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="F6" s="77" t="s">
+      <c r="F6" s="78" t="s">
         <v>139</v>
       </c>
-      <c r="G6" s="78"/>
-      <c r="H6" s="78"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="79"/>
       <c r="I6" s="23"/>
-      <c r="J6" s="80"/>
+      <c r="J6" s="81"/>
       <c r="K6" s="74"/>
       <c r="L6" s="20"/>
       <c r="M6" s="5"/>
     </row>
     <row r="7" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="81" t="s">
+      <c r="A7" s="73" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="74"/>
@@ -6668,7 +6668,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="74"/>
@@ -6767,26 +6767,26 @@
     <row r="6" spans="1:13" ht="151.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19"/>
       <c r="B6" s="19"/>
-      <c r="C6" s="79" t="s">
+      <c r="C6" s="80" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="78"/>
+      <c r="D6" s="79"/>
       <c r="E6" s="23" t="s">
         <v>174</v>
       </c>
-      <c r="F6" s="77" t="s">
+      <c r="F6" s="78" t="s">
         <v>175</v>
       </c>
-      <c r="G6" s="78"/>
-      <c r="H6" s="78"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="79"/>
       <c r="I6" s="23"/>
-      <c r="J6" s="80"/>
+      <c r="J6" s="81"/>
       <c r="K6" s="74"/>
       <c r="L6" s="20"/>
       <c r="M6" s="5"/>
     </row>
     <row r="7" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="81" t="s">
+      <c r="A7" s="73" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="74"/>
@@ -8285,7 +8285,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="74"/>
@@ -8384,26 +8384,26 @@
     <row r="6" spans="1:13" ht="151.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="19"/>
       <c r="B6" s="19"/>
-      <c r="C6" s="79" t="s">
+      <c r="C6" s="80" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="78"/>
+      <c r="D6" s="79"/>
       <c r="E6" s="23" t="s">
         <v>397</v>
       </c>
-      <c r="F6" s="77" t="s">
+      <c r="F6" s="78" t="s">
         <v>399</v>
       </c>
-      <c r="G6" s="78"/>
-      <c r="H6" s="78"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="79"/>
       <c r="I6" s="23"/>
-      <c r="J6" s="80"/>
+      <c r="J6" s="81"/>
       <c r="K6" s="74"/>
       <c r="L6" s="20"/>
       <c r="M6" s="5"/>
     </row>
     <row r="7" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="81" t="s">
+      <c r="A7" s="73" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="74"/>
@@ -8475,7 +8475,7 @@
         <v>402</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F10" s="28" t="s">
         <v>115</v>
@@ -8484,7 +8484,7 @@
         <v>46184</v>
       </c>
       <c r="H10" s="30" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="I10" s="22" t="s">
         <v>28</v>
@@ -9028,100 +9028,100 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:57" x14ac:dyDescent="0.25">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="84" t="s">
         <v>186</v>
       </c>
-      <c r="B1" s="85" t="s">
+      <c r="B1" s="84" t="s">
         <v>187</v>
       </c>
-      <c r="C1" s="85" t="s">
+      <c r="C1" s="84" t="s">
         <v>188</v>
       </c>
       <c r="D1" s="58" t="s">
         <v>159</v>
       </c>
-      <c r="E1" s="85" t="s">
+      <c r="E1" s="84" t="s">
         <v>189</v>
       </c>
-      <c r="F1" s="85" t="s">
+      <c r="F1" s="84" t="s">
         <v>190</v>
       </c>
-      <c r="G1" s="85" t="s">
+      <c r="G1" s="84" t="s">
         <v>191</v>
       </c>
-      <c r="H1" s="85" t="s">
+      <c r="H1" s="84" t="s">
         <v>192</v>
       </c>
-      <c r="I1" s="85" t="s">
+      <c r="I1" s="84" t="s">
         <v>193</v>
       </c>
-      <c r="J1" s="84" t="s">
+      <c r="J1" s="85" t="s">
         <v>194</v>
       </c>
       <c r="K1" s="74"/>
       <c r="L1" s="74"/>
       <c r="M1" s="74"/>
-      <c r="N1" s="84" t="s">
+      <c r="N1" s="85" t="s">
         <v>195</v>
       </c>
       <c r="O1" s="74"/>
       <c r="P1" s="74"/>
       <c r="Q1" s="74"/>
-      <c r="R1" s="84" t="s">
+      <c r="R1" s="85" t="s">
         <v>196</v>
       </c>
       <c r="S1" s="74"/>
       <c r="T1" s="74"/>
       <c r="U1" s="74"/>
-      <c r="V1" s="84" t="s">
+      <c r="V1" s="85" t="s">
         <v>197</v>
       </c>
       <c r="W1" s="74"/>
       <c r="X1" s="74"/>
       <c r="Y1" s="74"/>
-      <c r="Z1" s="84" t="s">
+      <c r="Z1" s="85" t="s">
         <v>198</v>
       </c>
       <c r="AA1" s="74"/>
       <c r="AB1" s="74"/>
       <c r="AC1" s="74"/>
-      <c r="AD1" s="84" t="s">
+      <c r="AD1" s="85" t="s">
         <v>199</v>
       </c>
       <c r="AE1" s="74"/>
       <c r="AF1" s="74"/>
       <c r="AG1" s="74"/>
-      <c r="AH1" s="84" t="s">
+      <c r="AH1" s="85" t="s">
         <v>200</v>
       </c>
       <c r="AI1" s="74"/>
       <c r="AJ1" s="74"/>
       <c r="AK1" s="74"/>
-      <c r="AL1" s="84" t="s">
+      <c r="AL1" s="85" t="s">
         <v>201</v>
       </c>
       <c r="AM1" s="74"/>
       <c r="AN1" s="74"/>
       <c r="AO1" s="74"/>
-      <c r="AP1" s="84" t="s">
+      <c r="AP1" s="85" t="s">
         <v>202</v>
       </c>
       <c r="AQ1" s="74"/>
       <c r="AR1" s="74"/>
       <c r="AS1" s="74"/>
-      <c r="AT1" s="84" t="s">
+      <c r="AT1" s="85" t="s">
         <v>203</v>
       </c>
       <c r="AU1" s="74"/>
       <c r="AV1" s="74"/>
       <c r="AW1" s="74"/>
-      <c r="AX1" s="84" t="s">
+      <c r="AX1" s="85" t="s">
         <v>204</v>
       </c>
       <c r="AY1" s="74"/>
       <c r="AZ1" s="74"/>
       <c r="BA1" s="74"/>
-      <c r="BB1" s="84" t="s">
+      <c r="BB1" s="85" t="s">
         <v>205</v>
       </c>
       <c r="BC1" s="74"/>
@@ -9134,10 +9134,10 @@
       <c r="C2" s="74"/>
       <c r="D2" s="58"/>
       <c r="E2" s="74"/>
-      <c r="F2" s="86"/>
+      <c r="F2" s="87"/>
       <c r="G2" s="74"/>
       <c r="H2" s="74"/>
-      <c r="I2" s="87"/>
+      <c r="I2" s="86"/>
       <c r="J2" s="39" t="s">
         <v>206</v>
       </c>
@@ -9289,10 +9289,10 @@
       <c r="C3" s="74"/>
       <c r="D3" s="58"/>
       <c r="E3" s="74"/>
-      <c r="F3" s="86"/>
+      <c r="F3" s="87"/>
       <c r="G3" s="74"/>
       <c r="H3" s="74"/>
-      <c r="I3" s="87"/>
+      <c r="I3" s="86"/>
       <c r="J3" s="39"/>
       <c r="K3" s="39"/>
       <c r="L3" s="39"/>
@@ -15545,6 +15545,15 @@
     <filterColumn colId="55" showButton="0"/>
   </autoFilter>
   <mergeCells count="20">
+    <mergeCell ref="BB1:BE1"/>
+    <mergeCell ref="F1:F3"/>
+    <mergeCell ref="R1:U1"/>
+    <mergeCell ref="AX1:BA1"/>
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="AP1:AS1"/>
+    <mergeCell ref="AH1:AK1"/>
+    <mergeCell ref="AL1:AO1"/>
+    <mergeCell ref="AT1:AW1"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="H1:H3"/>
     <mergeCell ref="V1:Y1"/>
@@ -15556,15 +15565,6 @@
     <mergeCell ref="G1:G3"/>
     <mergeCell ref="Z1:AC1"/>
     <mergeCell ref="I1:I3"/>
-    <mergeCell ref="BB1:BE1"/>
-    <mergeCell ref="F1:F3"/>
-    <mergeCell ref="R1:U1"/>
-    <mergeCell ref="AX1:BA1"/>
-    <mergeCell ref="J1:M1"/>
-    <mergeCell ref="AP1:AS1"/>
-    <mergeCell ref="AH1:AK1"/>
-    <mergeCell ref="AL1:AO1"/>
-    <mergeCell ref="AT1:AW1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>